<commit_message>
Visualització: a-Diagrama b-Network c-Coordenades. (a=graphviz, b, c=pyvis)
</commit_message>
<xml_diff>
--- a/data/network/edges.xlsx
+++ b/data/network/edges.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A425BF-FCCA-4DC7-B0C2-00472A696FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70792806-4AC9-4C81-8ED4-BEFA8C6537FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{306F75E9-4DFE-4518-8798-1CA0D2BB102C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="60">
   <si>
     <t>source</t>
   </si>
@@ -80,72 +80,24 @@
     <t>SS-2100/SS-2200</t>
   </si>
   <si>
-    <t>SS-2100/SS-2201</t>
-  </si>
-  <si>
-    <t>SS-2100/SS-2202</t>
-  </si>
-  <si>
-    <t>SS-2100/SS-2203</t>
-  </si>
-  <si>
     <t>SS-800</t>
   </si>
   <si>
     <t>SS-700B</t>
   </si>
   <si>
-    <t>Líquid-líquid</t>
-  </si>
-  <si>
     <t>P-600</t>
   </si>
   <si>
     <t>V-700/V-800</t>
   </si>
   <si>
-    <t>V-700/V-801</t>
-  </si>
-  <si>
-    <t>V-700/V-802</t>
-  </si>
-  <si>
-    <t>V-700/V-803</t>
-  </si>
-  <si>
-    <t>V-700/V-804</t>
-  </si>
-  <si>
     <t>E-900/E-1000</t>
   </si>
   <si>
-    <t>E-900/E-1001</t>
-  </si>
-  <si>
-    <t>E-900/E-1002</t>
-  </si>
-  <si>
-    <t>E-900/E-1003</t>
-  </si>
-  <si>
-    <t>E-900/E-1004</t>
-  </si>
-  <si>
-    <t>E-900/E-1005</t>
-  </si>
-  <si>
-    <t>E-900/E-1006</t>
-  </si>
-  <si>
     <t>E-800</t>
   </si>
   <si>
-    <t>E-801</t>
-  </si>
-  <si>
-    <t>E-802</t>
-  </si>
-  <si>
     <t>SIL-PEL</t>
   </si>
   <si>
@@ -264,6 +216,9 @@
   </si>
   <si>
     <t>cabal_teo-real</t>
+  </si>
+  <si>
+    <t>LIQ-LIQ</t>
   </si>
 </sst>
 </file>
@@ -644,10 +599,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9701035B-20B7-437C-B875-CAFA64730628}">
-  <dimension ref="A1:O89"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
     <col min="5" max="5" width="8.109375" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.33203125" customWidth="1"/>
     <col min="13" max="13" width="11.33203125" customWidth="1"/>
@@ -672,34 +627,34 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H1" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="I1" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="J1" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="K1" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="L1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="M1" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="N1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="O1" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -781,30 +736,30 @@
         <v>4.8</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I66" si="0">(G3-2*H3)*10^-3</f>
+        <f t="shared" ref="I3:I73" si="0">(G3-2*H3)*10^-3</f>
         <v>0.15870000000000001</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J66" si="1">PI()*I3^2/4</f>
+        <f t="shared" ref="J3:J73" si="1">PI()*I3^2/4</f>
         <v>1.9780794669897482E-2</v>
       </c>
       <c r="K3">
         <v>3</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:L66" si="2">J3*K3</f>
+        <f t="shared" ref="L3:L73" si="2">J3*K3</f>
         <v>5.9342384009692446E-2</v>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M66" si="3">L3*1000</f>
+        <f t="shared" ref="M3:M73" si="3">L3*1000</f>
         <v>59.342384009692445</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N66" si="4">L3*3600</f>
+        <f t="shared" ref="N3:N73" si="4">L3*3600</f>
         <v>213.63258243489281</v>
       </c>
       <c r="O3">
-        <f t="shared" ref="O3:O66" si="5">N3-C3</f>
+        <f t="shared" ref="O3:O73" si="5">N3-C3</f>
         <v>13.632582434892811</v>
       </c>
     </row>
@@ -981,7 +936,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F7">
         <v>350</v>
@@ -1034,7 +989,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F8">
         <v>350</v>
@@ -1087,7 +1042,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F9">
         <v>350</v>
@@ -1140,7 +1095,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F10">
         <v>350</v>
@@ -1193,7 +1148,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="F11">
         <v>350</v>
@@ -1246,7 +1201,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F12">
         <v>80</v>
@@ -1299,7 +1254,7 @@
         <v>6</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F13">
         <v>300</v>
@@ -1352,7 +1307,7 @@
         <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F14">
         <v>100</v>
@@ -1405,7 +1360,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F15">
         <v>300</v>
@@ -1458,7 +1413,7 @@
         <v>6</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="F16">
         <v>300</v>
@@ -1511,7 +1466,7 @@
         <v>6</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F17">
         <v>300</v>
@@ -1564,7 +1519,7 @@
         <v>6</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="F18">
         <v>300</v>
@@ -1617,7 +1572,7 @@
         <v>6</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="F19">
         <v>250</v>
@@ -1670,7 +1625,7 @@
         <v>6</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="F20">
         <v>200</v>
@@ -1723,7 +1678,7 @@
         <v>6</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="F21">
         <v>200</v>
@@ -1776,7 +1731,7 @@
         <v>6</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F22">
         <v>150</v>
@@ -1829,7 +1784,7 @@
         <v>6</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="F23">
         <v>150</v>
@@ -1882,7 +1837,7 @@
         <v>6</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="F24">
         <v>150</v>
@@ -1935,7 +1890,7 @@
         <v>6</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F25">
         <v>80</v>
@@ -1988,7 +1943,7 @@
         <v>6</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="F26">
         <v>80</v>
@@ -2041,7 +1996,7 @@
         <v>6</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F27">
         <v>80</v>
@@ -2094,7 +2049,7 @@
         <v>6</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="F28">
         <v>250</v>
@@ -2147,7 +2102,7 @@
         <v>6</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F29">
         <v>200</v>
@@ -2200,7 +2155,7 @@
         <v>6</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="F30">
         <v>200</v>
@@ -2253,7 +2208,7 @@
         <v>6</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="F31">
         <v>100</v>
@@ -2306,7 +2261,7 @@
         <v>6</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="F32">
         <v>100</v>
@@ -2356,7 +2311,7 @@
         <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E33" s="1">
         <v>51000</v>
@@ -2409,7 +2364,7 @@
         <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E34" s="1">
         <v>53000</v>
@@ -2838,6 +2793,9 @@
       <c r="E42" s="1">
         <v>1160.01</v>
       </c>
+      <c r="F42">
+        <v>204</v>
+      </c>
       <c r="G42">
         <v>204</v>
       </c>
@@ -2888,6 +2846,9 @@
       <c r="E43" s="1">
         <v>1160</v>
       </c>
+      <c r="F43">
+        <v>129</v>
+      </c>
       <c r="G43">
         <v>129</v>
       </c>
@@ -2938,6 +2899,9 @@
       <c r="E44" s="1">
         <v>1170</v>
       </c>
+      <c r="F44">
+        <v>100</v>
+      </c>
       <c r="G44">
         <v>114</v>
       </c>
@@ -3295,7 +3259,7 @@
         <v>23</v>
       </c>
       <c r="B51">
-        <v>5600</v>
+        <v>5600.01</v>
       </c>
       <c r="C51">
         <v>10</v>
@@ -3304,7 +3268,8 @@
         <v>9</v>
       </c>
       <c r="E51" s="1">
-        <v>5600</v>
+        <f>B51</f>
+        <v>5600.01</v>
       </c>
       <c r="F51">
         <v>80</v>
@@ -3345,431 +3310,431 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>24</v>
+        <v>5600.01</v>
       </c>
       <c r="B52">
-        <v>56000</v>
+        <v>5603</v>
       </c>
       <c r="C52">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D52" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E52" s="1">
-        <v>56000</v>
+        <f t="shared" ref="E52:E53" si="6">B52</f>
+        <v>5603</v>
       </c>
       <c r="F52">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G52">
-        <v>114</v>
+        <v>60.3</v>
       </c>
       <c r="H52">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="I52">
         <f t="shared" si="0"/>
-        <v>0.105</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J52">
         <f t="shared" si="1"/>
-        <v>8.6590147514568668E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K52">
         <v>1</v>
       </c>
       <c r="L52">
         <f t="shared" si="2"/>
-        <v>8.6590147514568668E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M52">
         <f t="shared" si="3"/>
-        <v>8.6590147514568674</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N52">
         <f t="shared" si="4"/>
-        <v>31.17245310524472</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O52">
         <f t="shared" si="5"/>
-        <v>26.17245310524472</v>
+        <v>-2.7740544210516305E-2</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>24</v>
+        <v>5600.01</v>
       </c>
       <c r="B53">
-        <v>52100.01</v>
+        <v>5601</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E53" s="1">
-        <v>52100.01</v>
+        <f t="shared" si="6"/>
+        <v>5601</v>
       </c>
       <c r="F53">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="G53">
-        <v>88.9</v>
+        <v>60.3</v>
       </c>
       <c r="H53">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="I53">
         <f t="shared" si="0"/>
-        <v>8.0900000000000014E-2</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J53">
         <f t="shared" si="1"/>
-        <v>5.1402817537852556E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K53">
         <v>1</v>
       </c>
       <c r="L53">
         <f t="shared" si="2"/>
-        <v>5.1402817537852556E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M53">
         <f t="shared" si="3"/>
-        <v>5.1402817537852554</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N53">
         <f t="shared" si="4"/>
-        <v>18.505014313626919</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O53">
         <f t="shared" si="5"/>
-        <v>18.505014313626919</v>
+        <v>5.9722594557894837</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>52100.01</v>
+        <v>24</v>
       </c>
       <c r="B54">
-        <v>52100.02</v>
+        <v>56000.01</v>
+      </c>
+      <c r="C54">
+        <v>5</v>
       </c>
       <c r="D54" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E54" s="1">
-        <v>52100.02</v>
+        <v>56000.01</v>
       </c>
       <c r="F54">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G54">
-        <v>88.9</v>
+        <v>114</v>
       </c>
       <c r="H54">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="I54">
         <f t="shared" si="0"/>
-        <v>8.0900000000000014E-2</v>
+        <v>0.105</v>
       </c>
       <c r="J54">
         <f t="shared" si="1"/>
-        <v>5.1402817537852556E-3</v>
+        <v>8.6590147514568668E-3</v>
       </c>
       <c r="K54">
         <v>1</v>
       </c>
       <c r="L54">
         <f t="shared" si="2"/>
-        <v>5.1402817537852556E-3</v>
+        <v>8.6590147514568668E-3</v>
       </c>
       <c r="M54">
         <f t="shared" si="3"/>
-        <v>5.1402817537852554</v>
+        <v>8.6590147514568674</v>
       </c>
       <c r="N54">
         <f t="shared" si="4"/>
-        <v>18.505014313626919</v>
+        <v>31.17245310524472</v>
       </c>
       <c r="O54">
         <f t="shared" si="5"/>
-        <v>18.505014313626919</v>
+        <v>26.17245310524472</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>52100.02</v>
+        <v>56000.01</v>
       </c>
       <c r="B55">
-        <v>52107</v>
+        <v>56002</v>
+      </c>
+      <c r="C55">
+        <v>5</v>
       </c>
       <c r="D55" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E55" s="1">
-        <v>52107</v>
+        <v>56002</v>
       </c>
       <c r="F55">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G55">
-        <v>76.099999999999994</v>
+        <v>60.3</v>
       </c>
       <c r="H55">
         <v>3.6</v>
       </c>
       <c r="I55">
         <f t="shared" si="0"/>
-        <v>6.8899999999999989E-2</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J55">
         <f t="shared" si="1"/>
-        <v>3.728450015261999E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K55">
         <v>1</v>
       </c>
       <c r="L55">
         <f t="shared" si="2"/>
-        <v>3.728450015261999E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M55">
         <f t="shared" si="3"/>
-        <v>3.7284500152619988</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N55">
         <f t="shared" si="4"/>
-        <v>13.422420054943197</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O55">
         <f t="shared" si="5"/>
-        <v>13.422420054943197</v>
+        <v>2.9722594557894837</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>52100.02</v>
+        <v>24</v>
       </c>
       <c r="B56">
-        <v>52207</v>
+        <v>52100.01</v>
       </c>
       <c r="D56" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E56" s="1">
-        <v>52207</v>
+        <v>52100.01</v>
       </c>
       <c r="F56">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G56">
-        <v>60.3</v>
+        <v>88.9</v>
       </c>
       <c r="H56">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="I56">
         <f t="shared" si="0"/>
-        <v>5.3099999999999994E-2</v>
+        <v>8.0900000000000014E-2</v>
       </c>
       <c r="J56">
         <f t="shared" si="1"/>
-        <v>2.2145165154970788E-3</v>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="K56">
         <v>1</v>
       </c>
       <c r="L56">
         <f t="shared" si="2"/>
-        <v>2.2145165154970788E-3</v>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="M56">
         <f t="shared" si="3"/>
-        <v>2.214516515497079</v>
+        <v>5.1402817537852554</v>
       </c>
       <c r="N56">
         <f t="shared" si="4"/>
-        <v>7.9722594557894837</v>
+        <v>18.505014313626919</v>
       </c>
       <c r="O56">
         <f t="shared" si="5"/>
-        <v>7.9722594557894837</v>
+        <v>18.505014313626919</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>7</v>
+        <v>52100.01</v>
       </c>
       <c r="B57">
-        <v>3700.01</v>
-      </c>
-      <c r="C57">
-        <v>100</v>
+        <v>52100.02</v>
       </c>
       <c r="D57" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E57" s="1">
-        <v>3700.01</v>
+        <v>52100.02</v>
       </c>
       <c r="F57">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="G57">
-        <v>220</v>
+        <v>88.9</v>
       </c>
       <c r="H57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I57">
         <f t="shared" si="0"/>
-        <v>0.21</v>
+        <v>8.0900000000000014E-2</v>
       </c>
       <c r="J57">
         <f t="shared" si="1"/>
-        <v>3.4636059005827467E-2</v>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="K57">
         <v>1</v>
       </c>
       <c r="L57">
         <f t="shared" si="2"/>
-        <v>3.4636059005827467E-2</v>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="M57">
         <f t="shared" si="3"/>
-        <v>34.63605900582747</v>
+        <v>5.1402817537852554</v>
       </c>
       <c r="N57">
         <f t="shared" si="4"/>
-        <v>124.68981242097888</v>
+        <v>18.505014313626919</v>
       </c>
       <c r="O57">
         <f t="shared" si="5"/>
-        <v>24.689812420978882</v>
+        <v>18.505014313626919</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>3700.01</v>
+        <v>52100.01</v>
       </c>
       <c r="B58">
-        <v>1120</v>
-      </c>
-      <c r="C58">
-        <v>100</v>
+        <v>52100.03</v>
       </c>
       <c r="D58" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E58" s="1">
-        <v>1120</v>
+        <f>B58</f>
+        <v>52100.03</v>
       </c>
       <c r="F58">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="G58">
-        <v>141</v>
+        <v>60.3</v>
       </c>
       <c r="H58">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="I58">
         <f t="shared" si="0"/>
-        <v>0.13100000000000001</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J58">
         <f t="shared" si="1"/>
-        <v>1.3478217882063612E-2</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K58">
         <v>1</v>
       </c>
       <c r="L58">
         <f t="shared" si="2"/>
-        <v>1.3478217882063612E-2</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M58">
         <f t="shared" si="3"/>
-        <v>13.478217882063612</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N58">
         <f t="shared" si="4"/>
-        <v>48.521584375429001</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O58">
         <f t="shared" si="5"/>
-        <v>-51.478415624570999</v>
+        <v>7.9722594557894837</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>13</v>
+        <v>52100.02</v>
       </c>
       <c r="B59">
-        <v>5800.01</v>
-      </c>
-      <c r="C59">
-        <v>100</v>
+        <v>52107</v>
       </c>
       <c r="D59" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E59" s="1">
-        <v>5800.01</v>
+        <v>52107</v>
       </c>
       <c r="F59">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="G59">
-        <v>114</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="H59">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="I59">
         <f t="shared" si="0"/>
-        <v>0.105</v>
+        <v>6.8899999999999989E-2</v>
       </c>
       <c r="J59">
         <f t="shared" si="1"/>
-        <v>8.6590147514568668E-3</v>
+        <v>3.728450015261999E-3</v>
       </c>
       <c r="K59">
         <v>1</v>
       </c>
       <c r="L59">
         <f t="shared" si="2"/>
-        <v>8.6590147514568668E-3</v>
+        <v>3.728450015261999E-3</v>
       </c>
       <c r="M59">
         <f t="shared" si="3"/>
-        <v>8.6590147514568674</v>
+        <v>3.7284500152619988</v>
       </c>
       <c r="N59">
         <f t="shared" si="4"/>
-        <v>31.17245310524472</v>
+        <v>13.422420054943197</v>
       </c>
       <c r="O59">
         <f t="shared" si="5"/>
-        <v>-68.827546894755272</v>
+        <v>13.422420054943197</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>5800.01</v>
+        <v>52100.02</v>
       </c>
       <c r="B60">
-        <v>5802</v>
-      </c>
-      <c r="C60">
-        <v>50</v>
+        <v>52207</v>
       </c>
       <c r="D60" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E60" s="1">
-        <v>5802</v>
+        <v>52207</v>
       </c>
       <c r="F60">
         <v>50</v>
@@ -3805,1518 +3770,1996 @@
       </c>
       <c r="O60">
         <f t="shared" si="5"/>
-        <v>-42.027740544210516</v>
+        <v>7.9722594557894837</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>5800.01</v>
+        <v>52100.03</v>
       </c>
       <c r="B61">
-        <v>5801</v>
-      </c>
-      <c r="C61">
+        <v>52100</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" s="1">
+        <f>B61</f>
+        <v>52100</v>
+      </c>
+      <c r="F61">
         <v>50</v>
       </c>
-      <c r="D61" t="s">
-        <v>16</v>
-      </c>
-      <c r="E61" s="1">
-        <v>5801</v>
-      </c>
-      <c r="F61">
-        <v>80</v>
-      </c>
       <c r="G61">
-        <v>88.9</v>
+        <v>60.3</v>
       </c>
       <c r="H61">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="I61">
         <f t="shared" si="0"/>
-        <v>8.0900000000000014E-2</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J61">
         <f t="shared" si="1"/>
-        <v>5.1402817537852556E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K61">
         <v>1</v>
       </c>
       <c r="L61">
         <f t="shared" si="2"/>
-        <v>5.1402817537852556E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M61">
         <f t="shared" si="3"/>
-        <v>5.1402817537852554</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N61">
         <f t="shared" si="4"/>
-        <v>18.505014313626919</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O61">
         <f t="shared" si="5"/>
-        <v>-31.494985686373081</v>
+        <v>7.9722594557894837</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>8</v>
+        <v>52100.03</v>
       </c>
       <c r="B62">
-        <v>5700.01</v>
-      </c>
-      <c r="C62">
-        <v>10</v>
+        <v>52200</v>
       </c>
       <c r="D62" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E62" s="1">
-        <v>5700.01</v>
+        <f>B62</f>
+        <v>52200</v>
       </c>
       <c r="F62">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G62">
-        <v>114</v>
+        <v>60.3</v>
       </c>
       <c r="H62">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="I62">
         <f t="shared" si="0"/>
-        <v>0.105</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J62">
         <f t="shared" si="1"/>
-        <v>8.6590147514568668E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K62">
         <v>1</v>
       </c>
       <c r="L62">
         <f t="shared" si="2"/>
-        <v>8.6590147514568668E-3</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M62">
         <f t="shared" si="3"/>
-        <v>8.6590147514568674</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N62">
         <f t="shared" si="4"/>
-        <v>31.17245310524472</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O62">
         <f t="shared" si="5"/>
-        <v>21.17245310524472</v>
+        <v>7.9722594557894837</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>5700.01</v>
+        <v>7</v>
       </c>
       <c r="B63">
-        <v>5701</v>
+        <v>3700.01</v>
       </c>
       <c r="C63">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D63" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E63" s="1">
-        <v>5701</v>
+        <v>3700.01</v>
       </c>
       <c r="F63">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="G63">
-        <v>88.9</v>
+        <v>220</v>
       </c>
       <c r="H63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I63">
         <f t="shared" si="0"/>
-        <v>8.0900000000000014E-2</v>
+        <v>0.21</v>
       </c>
       <c r="J63">
         <f t="shared" si="1"/>
-        <v>5.1402817537852556E-3</v>
+        <v>3.4636059005827467E-2</v>
       </c>
       <c r="K63">
         <v>1</v>
       </c>
       <c r="L63">
         <f t="shared" si="2"/>
-        <v>5.1402817537852556E-3</v>
+        <v>3.4636059005827467E-2</v>
       </c>
       <c r="M63">
         <f t="shared" si="3"/>
-        <v>5.1402817537852554</v>
+        <v>34.63605900582747</v>
       </c>
       <c r="N63">
         <f t="shared" si="4"/>
-        <v>18.505014313626919</v>
+        <v>124.68981242097888</v>
       </c>
       <c r="O63">
         <f t="shared" si="5"/>
-        <v>8.5050143136269192</v>
+        <v>24.689812420978882</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>12</v>
+        <v>3700.01</v>
       </c>
       <c r="B64">
-        <v>4600.01</v>
+        <v>1120</v>
       </c>
       <c r="C64">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D64" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E64" s="1">
-        <v>4600.01</v>
+        <v>1120</v>
       </c>
       <c r="F64">
-        <v>65</v>
+        <v>125</v>
       </c>
       <c r="G64">
-        <v>76.099999999999994</v>
+        <v>141</v>
       </c>
       <c r="H64">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="I64">
         <f t="shared" si="0"/>
-        <v>6.8899999999999989E-2</v>
+        <v>0.13100000000000001</v>
       </c>
       <c r="J64">
         <f t="shared" si="1"/>
-        <v>3.728450015261999E-3</v>
+        <v>1.3478217882063612E-2</v>
       </c>
       <c r="K64">
         <v>1</v>
       </c>
       <c r="L64">
         <f t="shared" si="2"/>
-        <v>3.728450015261999E-3</v>
+        <v>1.3478217882063612E-2</v>
       </c>
       <c r="M64">
         <f t="shared" si="3"/>
-        <v>3.7284500152619988</v>
+        <v>13.478217882063612</v>
       </c>
       <c r="N64">
         <f t="shared" si="4"/>
-        <v>13.422420054943197</v>
+        <v>48.521584375429001</v>
       </c>
       <c r="O64">
         <f t="shared" si="5"/>
-        <v>-1.5775799450568027</v>
+        <v>-51.478415624570999</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>4600.01</v>
+        <v>13</v>
       </c>
       <c r="B65">
-        <v>4671</v>
+        <v>5800.01</v>
       </c>
       <c r="C65">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D65" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E65" s="1">
-        <v>4671</v>
+        <v>5800.01</v>
       </c>
       <c r="F65">
-        <v>32</v>
+        <v>100</v>
       </c>
       <c r="G65">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="H65">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="I65">
         <f t="shared" si="0"/>
-        <v>3.6600000000000001E-2</v>
+        <v>0.105</v>
       </c>
       <c r="J65">
         <f t="shared" si="1"/>
-        <v>1.0520879637606858E-3</v>
+        <v>8.6590147514568668E-3</v>
       </c>
       <c r="K65">
         <v>1</v>
       </c>
       <c r="L65">
         <f t="shared" si="2"/>
-        <v>1.0520879637606858E-3</v>
+        <v>8.6590147514568668E-3</v>
       </c>
       <c r="M65">
         <f t="shared" si="3"/>
-        <v>1.0520879637606857</v>
+        <v>8.6590147514568674</v>
       </c>
       <c r="N65">
         <f t="shared" si="4"/>
-        <v>3.7875166695384688</v>
+        <v>31.17245310524472</v>
       </c>
       <c r="O65">
         <f t="shared" si="5"/>
-        <v>-11.212483330461531</v>
+        <v>-68.827546894755272</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>16</v>
+        <v>5800.01</v>
       </c>
       <c r="B66">
-        <v>4600.0200000000004</v>
+        <v>5802</v>
       </c>
       <c r="C66">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D66" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E66" s="1">
-        <v>4600.0200000000004</v>
+        <v>5802</v>
       </c>
       <c r="F66">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="G66">
-        <v>139.69999999999999</v>
+        <v>60.3</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="I66">
         <f t="shared" si="0"/>
-        <v>0.12969999999999998</v>
+        <v>5.3099999999999994E-2</v>
       </c>
       <c r="J66">
         <f t="shared" si="1"/>
-        <v>1.3212038590506577E-2</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="K66">
         <v>1</v>
       </c>
       <c r="L66">
         <f t="shared" si="2"/>
-        <v>1.3212038590506577E-2</v>
+        <v>2.2145165154970788E-3</v>
       </c>
       <c r="M66">
         <f t="shared" si="3"/>
-        <v>13.212038590506577</v>
+        <v>2.214516515497079</v>
       </c>
       <c r="N66">
         <f t="shared" si="4"/>
-        <v>47.563338925823679</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="O66">
         <f t="shared" si="5"/>
-        <v>22.563338925823679</v>
+        <v>-42.027740544210516</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>4600.0200000000004</v>
+        <v>5800.01</v>
       </c>
       <c r="B67">
-        <v>4651</v>
+        <v>5801</v>
       </c>
       <c r="C67">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E67" s="1">
-        <v>4651</v>
+        <v>5801</v>
       </c>
       <c r="F67">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G67">
-        <v>60.3</v>
+        <v>88.9</v>
       </c>
       <c r="H67">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="I67">
-        <f t="shared" ref="I67:I89" si="6">(G67-2*H67)*10^-3</f>
-        <v>5.3099999999999994E-2</v>
+        <f t="shared" si="0"/>
+        <v>8.0900000000000014E-2</v>
       </c>
       <c r="J67">
-        <f t="shared" ref="J67:J89" si="7">PI()*I67^2/4</f>
-        <v>2.2145165154970788E-3</v>
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="K67">
         <v>1</v>
       </c>
       <c r="L67">
-        <f t="shared" ref="L67:L89" si="8">J67*K67</f>
-        <v>2.2145165154970788E-3</v>
+        <f t="shared" si="2"/>
+        <v>5.1402817537852556E-3</v>
       </c>
       <c r="M67">
-        <f t="shared" ref="M67:M89" si="9">L67*1000</f>
-        <v>2.214516515497079</v>
+        <f t="shared" si="3"/>
+        <v>5.1402817537852554</v>
       </c>
       <c r="N67">
-        <f t="shared" ref="N67:N89" si="10">L67*3600</f>
-        <v>7.9722594557894837</v>
+        <f t="shared" si="4"/>
+        <v>18.505014313626919</v>
       </c>
       <c r="O67">
-        <f t="shared" ref="O67:O89" si="11">N67-C67</f>
-        <v>-17.027740544210516</v>
+        <f t="shared" si="5"/>
+        <v>-31.494985686373081</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B68">
-        <v>4501</v>
+        <v>5700.01</v>
       </c>
       <c r="C68">
         <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E68" s="1">
+        <v>5700.01</v>
+      </c>
+      <c r="F68">
+        <v>100</v>
+      </c>
+      <c r="G68">
+        <v>114</v>
+      </c>
+      <c r="H68">
+        <v>4.5</v>
+      </c>
+      <c r="I68">
+        <f t="shared" si="0"/>
+        <v>0.105</v>
+      </c>
+      <c r="J68">
+        <f t="shared" si="1"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="K68">
+        <v>1</v>
+      </c>
+      <c r="L68">
+        <f t="shared" si="2"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="M68">
+        <f t="shared" si="3"/>
+        <v>8.6590147514568674</v>
+      </c>
+      <c r="N68">
+        <f t="shared" si="4"/>
+        <v>31.17245310524472</v>
+      </c>
+      <c r="O68">
+        <f t="shared" si="5"/>
+        <v>21.17245310524472</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>5700.01</v>
+      </c>
+      <c r="B69">
+        <v>5701</v>
+      </c>
+      <c r="C69">
+        <v>10</v>
+      </c>
+      <c r="D69" t="s">
+        <v>14</v>
+      </c>
+      <c r="E69" s="1">
+        <v>5701</v>
+      </c>
+      <c r="F69">
+        <v>80</v>
+      </c>
+      <c r="G69">
+        <v>88.9</v>
+      </c>
+      <c r="H69">
+        <v>4</v>
+      </c>
+      <c r="I69">
+        <f t="shared" si="0"/>
+        <v>8.0900000000000014E-2</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="K69">
+        <v>1</v>
+      </c>
+      <c r="L69">
+        <f t="shared" si="2"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="M69">
+        <f t="shared" si="3"/>
+        <v>5.1402817537852554</v>
+      </c>
+      <c r="N69">
+        <f t="shared" si="4"/>
+        <v>18.505014313626919</v>
+      </c>
+      <c r="O69">
+        <f t="shared" si="5"/>
+        <v>8.5050143136269192</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>12</v>
+      </c>
+      <c r="B70">
+        <v>4600.01</v>
+      </c>
+      <c r="C70">
+        <v>15</v>
+      </c>
+      <c r="D70" t="s">
+        <v>59</v>
+      </c>
+      <c r="E70" s="1">
+        <v>4600.01</v>
+      </c>
+      <c r="F70">
+        <v>65</v>
+      </c>
+      <c r="G70">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="H70">
+        <v>3.6</v>
+      </c>
+      <c r="I70">
+        <f t="shared" si="0"/>
+        <v>6.8899999999999989E-2</v>
+      </c>
+      <c r="J70">
+        <f t="shared" si="1"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="K70">
+        <v>1</v>
+      </c>
+      <c r="L70">
+        <f t="shared" si="2"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M70">
+        <f t="shared" si="3"/>
+        <v>3.7284500152619988</v>
+      </c>
+      <c r="N70">
+        <f t="shared" si="4"/>
+        <v>13.422420054943197</v>
+      </c>
+      <c r="O70">
+        <f t="shared" si="5"/>
+        <v>-1.5775799450568027</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>4600.01</v>
+      </c>
+      <c r="B71">
+        <v>4671</v>
+      </c>
+      <c r="C71">
+        <v>15</v>
+      </c>
+      <c r="D71" t="s">
+        <v>59</v>
+      </c>
+      <c r="E71" s="1">
+        <v>4671</v>
+      </c>
+      <c r="F71">
+        <v>32</v>
+      </c>
+      <c r="G71">
+        <v>43</v>
+      </c>
+      <c r="H71">
+        <v>3.2</v>
+      </c>
+      <c r="I71">
+        <f t="shared" si="0"/>
+        <v>3.6600000000000001E-2</v>
+      </c>
+      <c r="J71">
+        <f t="shared" si="1"/>
+        <v>1.0520879637606858E-3</v>
+      </c>
+      <c r="K71">
+        <v>1</v>
+      </c>
+      <c r="L71">
+        <f t="shared" si="2"/>
+        <v>1.0520879637606858E-3</v>
+      </c>
+      <c r="M71">
+        <f t="shared" si="3"/>
+        <v>1.0520879637606857</v>
+      </c>
+      <c r="N71">
+        <f t="shared" si="4"/>
+        <v>3.7875166695384688</v>
+      </c>
+      <c r="O71">
+        <f t="shared" si="5"/>
+        <v>-11.212483330461531</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>4600.01</v>
+      </c>
+      <c r="B72">
+        <v>4670</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+      <c r="D72" t="s">
+        <v>59</v>
+      </c>
+      <c r="E72" s="1">
+        <v>4670</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>16</v>
+      </c>
+      <c r="B73">
+        <v>4600.0200000000004</v>
+      </c>
+      <c r="C73">
+        <v>25</v>
+      </c>
+      <c r="D73" t="s">
+        <v>59</v>
+      </c>
+      <c r="E73" s="1">
+        <v>4600.0200000000004</v>
+      </c>
+      <c r="F73">
+        <v>125</v>
+      </c>
+      <c r="G73">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="H73">
+        <v>5</v>
+      </c>
+      <c r="I73">
+        <f t="shared" si="0"/>
+        <v>0.12969999999999998</v>
+      </c>
+      <c r="J73">
+        <f t="shared" si="1"/>
+        <v>1.3212038590506577E-2</v>
+      </c>
+      <c r="K73">
+        <v>1</v>
+      </c>
+      <c r="L73">
+        <f t="shared" si="2"/>
+        <v>1.3212038590506577E-2</v>
+      </c>
+      <c r="M73">
+        <f t="shared" si="3"/>
+        <v>13.212038590506577</v>
+      </c>
+      <c r="N73">
+        <f t="shared" si="4"/>
+        <v>47.563338925823679</v>
+      </c>
+      <c r="O73">
+        <f t="shared" si="5"/>
+        <v>22.563338925823679</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>4600.0200000000004</v>
+      </c>
+      <c r="B74">
+        <v>4651</v>
+      </c>
+      <c r="C74">
+        <v>25</v>
+      </c>
+      <c r="D74" t="s">
+        <v>59</v>
+      </c>
+      <c r="E74" s="1">
+        <v>4651</v>
+      </c>
+      <c r="F74">
+        <v>50</v>
+      </c>
+      <c r="G74">
+        <v>60.3</v>
+      </c>
+      <c r="H74">
+        <v>3.6</v>
+      </c>
+      <c r="I74">
+        <f t="shared" ref="I74:I98" si="7">(G74-2*H74)*10^-3</f>
+        <v>5.3099999999999994E-2</v>
+      </c>
+      <c r="J74">
+        <f t="shared" ref="J74:J98" si="8">PI()*I74^2/4</f>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="K74">
+        <v>1</v>
+      </c>
+      <c r="L74">
+        <f t="shared" ref="L74:L98" si="9">J74*K74</f>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M74">
+        <f t="shared" ref="M74:M98" si="10">L74*1000</f>
+        <v>2.214516515497079</v>
+      </c>
+      <c r="N74">
+        <f t="shared" ref="N74:N98" si="11">L74*3600</f>
+        <v>7.9722594557894837</v>
+      </c>
+      <c r="O74">
+        <f t="shared" ref="O74:O98" si="12">N74-C74</f>
+        <v>-17.027740544210516</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>17</v>
+      </c>
+      <c r="B75">
         <v>4501</v>
       </c>
-      <c r="F68">
+      <c r="C75">
+        <v>10</v>
+      </c>
+      <c r="D75" t="s">
+        <v>15</v>
+      </c>
+      <c r="E75" s="1">
+        <v>4501</v>
+      </c>
+      <c r="F75">
         <v>50</v>
       </c>
-      <c r="G68">
+      <c r="G75">
         <v>60.3</v>
       </c>
-      <c r="H68">
+      <c r="H75">
         <v>3.6</v>
       </c>
-      <c r="I68">
-        <f t="shared" si="6"/>
+      <c r="I75">
+        <f t="shared" si="7"/>
         <v>5.3099999999999994E-2</v>
       </c>
-      <c r="J68">
-        <f t="shared" si="7"/>
-        <v>2.2145165154970788E-3</v>
-      </c>
-      <c r="K68">
-        <v>1</v>
-      </c>
-      <c r="L68">
+      <c r="J75">
         <f t="shared" si="8"/>
         <v>2.2145165154970788E-3</v>
       </c>
-      <c r="M68">
+      <c r="K75">
+        <v>1</v>
+      </c>
+      <c r="L75">
         <f t="shared" si="9"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M75">
+        <f t="shared" si="10"/>
         <v>2.214516515497079</v>
       </c>
-      <c r="N68">
-        <f t="shared" si="10"/>
+      <c r="N75">
+        <f t="shared" si="11"/>
         <v>7.9722594557894837</v>
       </c>
-      <c r="O68">
-        <f t="shared" si="11"/>
+      <c r="O75">
+        <f t="shared" si="12"/>
         <v>-2.0277405442105163</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A76">
         <v>9</v>
       </c>
-      <c r="B69">
+      <c r="B76">
         <v>4700.01</v>
       </c>
-      <c r="C69">
+      <c r="C76">
         <v>50</v>
       </c>
-      <c r="D69" t="s">
-        <v>20</v>
-      </c>
-      <c r="E69" s="1">
+      <c r="D76" t="s">
+        <v>16</v>
+      </c>
+      <c r="E76" s="1">
         <v>4700.01</v>
       </c>
-      <c r="F69">
+      <c r="F76">
         <v>150</v>
       </c>
-      <c r="G69">
+      <c r="G76">
         <v>168.3</v>
       </c>
-      <c r="H69">
+      <c r="H76">
         <v>5</v>
       </c>
-      <c r="I69">
-        <f t="shared" si="6"/>
+      <c r="I76">
+        <f t="shared" si="7"/>
         <v>0.15830000000000002</v>
       </c>
-      <c r="J69">
-        <f t="shared" si="7"/>
-        <v>1.9681206182778688E-2</v>
-      </c>
-      <c r="K69">
-        <v>1</v>
-      </c>
-      <c r="L69">
+      <c r="J76">
         <f t="shared" si="8"/>
         <v>1.9681206182778688E-2</v>
       </c>
-      <c r="M69">
+      <c r="K76">
+        <v>1</v>
+      </c>
+      <c r="L76">
         <f t="shared" si="9"/>
+        <v>1.9681206182778688E-2</v>
+      </c>
+      <c r="M76">
+        <f t="shared" si="10"/>
         <v>19.681206182778688</v>
       </c>
-      <c r="N69">
-        <f t="shared" si="10"/>
+      <c r="N76">
+        <f t="shared" si="11"/>
         <v>70.852342258003276</v>
       </c>
-      <c r="O69">
-        <f t="shared" si="11"/>
+      <c r="O76">
+        <f t="shared" si="12"/>
         <v>20.852342258003276</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A77">
         <v>4700.01</v>
       </c>
-      <c r="B70">
+      <c r="B77">
         <v>4700.0200000000004</v>
       </c>
-      <c r="C70">
+      <c r="C77">
         <v>40</v>
       </c>
-      <c r="D70" t="s">
-        <v>21</v>
-      </c>
-      <c r="E70" s="1">
+      <c r="D77" t="s">
+        <v>16</v>
+      </c>
+      <c r="E77" s="1">
         <v>4700.0200000000004</v>
       </c>
-      <c r="F70">
+      <c r="F77">
         <v>100</v>
       </c>
-      <c r="G70">
+      <c r="G77">
         <v>114</v>
       </c>
-      <c r="H70">
+      <c r="H77">
         <v>4.5</v>
       </c>
-      <c r="I70">
-        <f t="shared" si="6"/>
+      <c r="I77">
+        <f t="shared" si="7"/>
         <v>0.105</v>
       </c>
-      <c r="J70">
-        <f t="shared" si="7"/>
-        <v>8.6590147514568668E-3</v>
-      </c>
-      <c r="K70">
-        <v>1</v>
-      </c>
-      <c r="L70">
+      <c r="J77">
         <f t="shared" si="8"/>
         <v>8.6590147514568668E-3</v>
       </c>
-      <c r="M70">
+      <c r="K77">
+        <v>1</v>
+      </c>
+      <c r="L77">
         <f t="shared" si="9"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="M77">
+        <f t="shared" si="10"/>
         <v>8.6590147514568674</v>
       </c>
-      <c r="N70">
-        <f t="shared" si="10"/>
+      <c r="N77">
+        <f t="shared" si="11"/>
         <v>31.17245310524472</v>
       </c>
-      <c r="O70">
-        <f t="shared" si="11"/>
+      <c r="O77">
+        <f t="shared" si="12"/>
         <v>-8.8275468947552795</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A78">
         <v>4700.0200000000004</v>
       </c>
-      <c r="B71">
+      <c r="B78">
         <v>4810</v>
       </c>
-      <c r="C71">
+      <c r="C78">
         <v>20</v>
       </c>
-      <c r="D71" t="s">
-        <v>22</v>
-      </c>
-      <c r="E71" s="1">
+      <c r="D78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E78" s="1">
         <v>4810</v>
       </c>
-      <c r="F71">
+      <c r="F78">
         <v>65</v>
       </c>
-      <c r="G71">
+      <c r="G78">
         <v>76.099999999999994</v>
       </c>
-      <c r="H71">
+      <c r="H78">
         <v>3.6</v>
       </c>
-      <c r="I71">
-        <f t="shared" si="6"/>
+      <c r="I78">
+        <f t="shared" si="7"/>
         <v>6.8899999999999989E-2</v>
       </c>
-      <c r="J71">
-        <f t="shared" si="7"/>
-        <v>3.728450015261999E-3</v>
-      </c>
-      <c r="K71">
-        <v>1</v>
-      </c>
-      <c r="L71">
+      <c r="J78">
         <f t="shared" si="8"/>
         <v>3.728450015261999E-3</v>
       </c>
-      <c r="M71">
+      <c r="K78">
+        <v>1</v>
+      </c>
+      <c r="L78">
         <f t="shared" si="9"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M78">
+        <f t="shared" si="10"/>
         <v>3.7284500152619988</v>
       </c>
-      <c r="N71">
-        <f t="shared" si="10"/>
+      <c r="N78">
+        <f t="shared" si="11"/>
         <v>13.422420054943197</v>
       </c>
-      <c r="O71">
-        <f t="shared" si="11"/>
+      <c r="O78">
+        <f t="shared" si="12"/>
         <v>-6.5775799450568027</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A79">
         <v>4700.0200000000004</v>
       </c>
-      <c r="B72">
+      <c r="B79">
         <v>4710</v>
       </c>
-      <c r="C72">
+      <c r="C79">
         <v>20</v>
       </c>
-      <c r="D72" t="s">
-        <v>23</v>
-      </c>
-      <c r="E72" s="1">
+      <c r="D79" t="s">
+        <v>16</v>
+      </c>
+      <c r="E79" s="1">
         <v>4710</v>
       </c>
-      <c r="F72">
+      <c r="F79">
         <v>65</v>
       </c>
-      <c r="G72">
+      <c r="G79">
         <v>76.099999999999994</v>
       </c>
-      <c r="H72">
+      <c r="H79">
         <v>3.6</v>
       </c>
-      <c r="I72">
-        <f t="shared" si="6"/>
+      <c r="I79">
+        <f t="shared" si="7"/>
         <v>6.8899999999999989E-2</v>
       </c>
-      <c r="J72">
-        <f t="shared" si="7"/>
-        <v>3.728450015261999E-3</v>
-      </c>
-      <c r="K72">
-        <v>1</v>
-      </c>
-      <c r="L72">
+      <c r="J79">
         <f t="shared" si="8"/>
         <v>3.728450015261999E-3</v>
       </c>
-      <c r="M72">
+      <c r="K79">
+        <v>1</v>
+      </c>
+      <c r="L79">
         <f t="shared" si="9"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M79">
+        <f t="shared" si="10"/>
         <v>3.7284500152619988</v>
       </c>
-      <c r="N72">
-        <f t="shared" si="10"/>
+      <c r="N79">
+        <f t="shared" si="11"/>
         <v>13.422420054943197</v>
       </c>
-      <c r="O72">
-        <f t="shared" si="11"/>
+      <c r="O79">
+        <f t="shared" si="12"/>
         <v>-6.5775799450568027</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A73">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A80">
         <v>4700.01</v>
       </c>
-      <c r="B73">
+      <c r="B80">
         <v>4740</v>
       </c>
-      <c r="C73">
+      <c r="C80">
         <v>10</v>
       </c>
-      <c r="D73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E73" s="1">
+      <c r="D80" t="s">
+        <v>16</v>
+      </c>
+      <c r="E80" s="1">
         <v>4740</v>
       </c>
-      <c r="F73">
+      <c r="F80">
         <v>25</v>
       </c>
-      <c r="G73">
+      <c r="G80">
         <v>33.700000000000003</v>
       </c>
-      <c r="H73">
+      <c r="H80">
         <v>3.2</v>
       </c>
-      <c r="I73">
-        <f t="shared" si="6"/>
+      <c r="I80">
+        <f t="shared" si="7"/>
         <v>2.7300000000000005E-2</v>
       </c>
-      <c r="J73">
-        <f t="shared" si="7"/>
-        <v>5.8534939719848437E-4</v>
-      </c>
-      <c r="K73">
-        <v>1</v>
-      </c>
-      <c r="L73">
+      <c r="J80">
         <f t="shared" si="8"/>
         <v>5.8534939719848437E-4</v>
       </c>
-      <c r="M73">
+      <c r="K80">
+        <v>1</v>
+      </c>
+      <c r="L80">
         <f t="shared" si="9"/>
+        <v>5.8534939719848437E-4</v>
+      </c>
+      <c r="M80">
+        <f t="shared" si="10"/>
         <v>0.58534939719848433</v>
       </c>
-      <c r="N73">
-        <f t="shared" si="10"/>
+      <c r="N80">
+        <f t="shared" si="11"/>
         <v>2.1072578299145439</v>
       </c>
-      <c r="O73">
-        <f t="shared" si="11"/>
+      <c r="O80">
+        <f t="shared" si="12"/>
         <v>-7.8927421700854561</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A74">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>4700.0200000000004</v>
+      </c>
+      <c r="B81">
+        <v>4711</v>
+      </c>
+      <c r="C81">
+        <v>0</v>
+      </c>
+      <c r="D81" t="s">
+        <v>16</v>
+      </c>
+      <c r="E81">
+        <v>4711</v>
+      </c>
+      <c r="F81">
+        <v>50</v>
+      </c>
+      <c r="G81">
+        <v>60.3</v>
+      </c>
+      <c r="H81">
+        <v>3.6</v>
+      </c>
+      <c r="I81">
+        <f t="shared" si="7"/>
+        <v>5.3099999999999994E-2</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="8"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="K81">
+        <v>1</v>
+      </c>
+      <c r="L81">
+        <f t="shared" ref="L81:L82" si="13">J81*K81</f>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M81">
+        <f t="shared" ref="M81:M82" si="14">L81*1000</f>
+        <v>2.214516515497079</v>
+      </c>
+      <c r="N81">
+        <f t="shared" ref="N81:N82" si="15">L81*3600</f>
+        <v>7.9722594557894837</v>
+      </c>
+      <c r="O81">
+        <f t="shared" ref="O81:O82" si="16">N81-C81</f>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>4700.0200000000004</v>
+      </c>
+      <c r="B82">
+        <v>4811</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+      <c r="D82" t="s">
+        <v>16</v>
+      </c>
+      <c r="E82">
+        <v>4811</v>
+      </c>
+      <c r="F82">
+        <v>50</v>
+      </c>
+      <c r="G82">
+        <v>60.3</v>
+      </c>
+      <c r="H82">
+        <v>3.6</v>
+      </c>
+      <c r="I82">
+        <f t="shared" si="7"/>
+        <v>5.3099999999999994E-2</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="8"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="K82">
+        <v>1</v>
+      </c>
+      <c r="L82">
+        <f t="shared" si="13"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M82">
+        <f t="shared" si="14"/>
+        <v>2.214516515497079</v>
+      </c>
+      <c r="N82">
+        <f t="shared" si="15"/>
+        <v>7.9722594557894837</v>
+      </c>
+      <c r="O82">
+        <f t="shared" si="16"/>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A83">
         <v>10</v>
       </c>
-      <c r="B74">
+      <c r="B83">
         <v>3900.01</v>
       </c>
-      <c r="C74">
+      <c r="C83">
         <v>300</v>
       </c>
-      <c r="D74" t="s">
-        <v>25</v>
-      </c>
-      <c r="E74" s="1">
+      <c r="D83" t="s">
+        <v>17</v>
+      </c>
+      <c r="E83" s="1">
         <v>3900.01</v>
       </c>
-      <c r="G74">
+      <c r="F83">
+        <f>G83</f>
         <v>204</v>
       </c>
-      <c r="H74">
+      <c r="G83">
+        <v>204</v>
+      </c>
+      <c r="H83">
         <v>2</v>
       </c>
-      <c r="I74">
-        <f t="shared" si="6"/>
+      <c r="I83">
+        <f t="shared" si="7"/>
         <v>0.2</v>
       </c>
-      <c r="J74">
-        <f t="shared" si="7"/>
-        <v>3.1415926535897934E-2</v>
-      </c>
-      <c r="K74">
-        <v>1</v>
-      </c>
-      <c r="L74">
+      <c r="J83">
         <f t="shared" si="8"/>
         <v>3.1415926535897934E-2</v>
       </c>
-      <c r="M74">
+      <c r="K83">
+        <v>1</v>
+      </c>
+      <c r="L83">
         <f t="shared" si="9"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="M83">
+        <f t="shared" si="10"/>
         <v>31.415926535897935</v>
       </c>
-      <c r="N74">
-        <f t="shared" si="10"/>
+      <c r="N83">
+        <f t="shared" si="11"/>
         <v>113.09733552923257</v>
       </c>
-      <c r="O74">
-        <f t="shared" si="11"/>
+      <c r="O83">
+        <f t="shared" si="12"/>
         <v>-186.90266447076743</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A75">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A84">
         <v>3900.01</v>
       </c>
-      <c r="B75">
+      <c r="B84">
         <v>3900.02</v>
       </c>
-      <c r="C75">
+      <c r="C84">
         <v>200</v>
       </c>
-      <c r="D75" t="s">
-        <v>26</v>
-      </c>
-      <c r="E75" s="1">
+      <c r="D84" t="s">
+        <v>17</v>
+      </c>
+      <c r="E84" s="1">
         <v>3900.02</v>
       </c>
-      <c r="G75">
+      <c r="F84">
+        <f t="shared" ref="F84:F92" si="17">G84</f>
         <v>204</v>
       </c>
-      <c r="H75">
+      <c r="G84">
+        <v>204</v>
+      </c>
+      <c r="H84">
         <v>2</v>
       </c>
-      <c r="I75">
-        <f t="shared" si="6"/>
+      <c r="I84">
+        <f t="shared" si="7"/>
         <v>0.2</v>
       </c>
-      <c r="J75">
-        <f t="shared" si="7"/>
-        <v>3.1415926535897934E-2</v>
-      </c>
-      <c r="K75">
-        <v>1</v>
-      </c>
-      <c r="L75">
+      <c r="J84">
         <f t="shared" si="8"/>
         <v>3.1415926535897934E-2</v>
       </c>
-      <c r="M75">
+      <c r="K84">
+        <v>1</v>
+      </c>
+      <c r="L84">
         <f t="shared" si="9"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="M84">
+        <f t="shared" si="10"/>
         <v>31.415926535897935</v>
       </c>
-      <c r="N75">
-        <f t="shared" si="10"/>
+      <c r="N84">
+        <f t="shared" si="11"/>
         <v>113.09733552923257</v>
       </c>
-      <c r="O75">
-        <f t="shared" si="11"/>
+      <c r="O84">
+        <f t="shared" si="12"/>
         <v>-86.902664470767434</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A76">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A85">
         <v>3900.02</v>
       </c>
-      <c r="B76">
+      <c r="B85">
         <v>3900.03</v>
       </c>
-      <c r="C76">
+      <c r="C85">
         <v>100</v>
       </c>
-      <c r="D76" t="s">
-        <v>27</v>
-      </c>
-      <c r="E76" s="1">
+      <c r="D85" t="s">
+        <v>17</v>
+      </c>
+      <c r="E85" s="1">
         <v>3900.03</v>
       </c>
-      <c r="G76">
+      <c r="F85">
+        <f t="shared" si="17"/>
         <v>155</v>
       </c>
-      <c r="H76">
+      <c r="G85">
+        <v>155</v>
+      </c>
+      <c r="H85">
         <v>2</v>
       </c>
-      <c r="I76">
-        <f t="shared" si="6"/>
+      <c r="I85">
+        <f t="shared" si="7"/>
         <v>0.151</v>
       </c>
-      <c r="J76">
-        <f t="shared" si="7"/>
-        <v>1.7907863523625216E-2</v>
-      </c>
-      <c r="K76">
-        <v>1</v>
-      </c>
-      <c r="L76">
+      <c r="J85">
         <f t="shared" si="8"/>
         <v>1.7907863523625216E-2</v>
       </c>
-      <c r="M76">
+      <c r="K85">
+        <v>1</v>
+      </c>
+      <c r="L85">
         <f t="shared" si="9"/>
+        <v>1.7907863523625216E-2</v>
+      </c>
+      <c r="M85">
+        <f t="shared" si="10"/>
         <v>17.907863523625217</v>
       </c>
-      <c r="N76">
-        <f t="shared" si="10"/>
+      <c r="N85">
+        <f t="shared" si="11"/>
         <v>64.468308685050772</v>
       </c>
-      <c r="O76">
-        <f t="shared" si="11"/>
+      <c r="O85">
+        <f t="shared" si="12"/>
         <v>-35.531691314949228</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A77">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A86">
         <v>3900.01</v>
       </c>
-      <c r="B77">
+      <c r="B86">
         <v>31001</v>
       </c>
-      <c r="C77">
+      <c r="C86">
         <v>100</v>
       </c>
-      <c r="D77" t="s">
-        <v>28</v>
-      </c>
-      <c r="E77" s="1">
+      <c r="D86" t="s">
+        <v>17</v>
+      </c>
+      <c r="E86" s="1">
         <v>31001</v>
       </c>
-      <c r="G77">
+      <c r="F86">
+        <f t="shared" si="17"/>
         <v>88.9</v>
       </c>
-      <c r="H77">
+      <c r="G86">
+        <v>88.9</v>
+      </c>
+      <c r="H86">
         <v>2</v>
       </c>
-      <c r="I77">
-        <f t="shared" si="6"/>
+      <c r="I86">
+        <f t="shared" si="7"/>
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="J77">
-        <f t="shared" si="7"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="K77">
-        <v>1</v>
-      </c>
-      <c r="L77">
+      <c r="J86">
         <f t="shared" si="8"/>
         <v>5.661157815750442E-3</v>
       </c>
-      <c r="M77">
+      <c r="K86">
+        <v>1</v>
+      </c>
+      <c r="L86">
         <f t="shared" si="9"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="M86">
+        <f t="shared" si="10"/>
         <v>5.6611578157504416</v>
       </c>
-      <c r="N77">
-        <f t="shared" si="10"/>
+      <c r="N86">
+        <f t="shared" si="11"/>
         <v>20.380168136701592</v>
       </c>
-      <c r="O77">
-        <f t="shared" si="11"/>
+      <c r="O86">
+        <f t="shared" si="12"/>
         <v>-79.619831863298401</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A78">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A87">
         <v>3900.02</v>
       </c>
-      <c r="B78">
+      <c r="B87">
         <v>3901</v>
       </c>
-      <c r="C78">
+      <c r="C87">
         <v>100</v>
       </c>
-      <c r="D78" t="s">
-        <v>29</v>
-      </c>
-      <c r="E78" s="1">
+      <c r="D87" t="s">
+        <v>17</v>
+      </c>
+      <c r="E87" s="1">
         <v>3901</v>
       </c>
-      <c r="G78">
+      <c r="F87">
+        <f t="shared" si="17"/>
         <v>88.9</v>
       </c>
-      <c r="H78">
+      <c r="G87">
+        <v>88.9</v>
+      </c>
+      <c r="H87">
         <v>2</v>
       </c>
-      <c r="I78">
-        <f t="shared" si="6"/>
+      <c r="I87">
+        <f t="shared" si="7"/>
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="J78">
-        <f t="shared" si="7"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="K78">
-        <v>1</v>
-      </c>
-      <c r="L78">
+      <c r="J87">
         <f t="shared" si="8"/>
         <v>5.661157815750442E-3</v>
       </c>
-      <c r="M78">
+      <c r="K87">
+        <v>1</v>
+      </c>
+      <c r="L87">
         <f t="shared" si="9"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="M87">
+        <f t="shared" si="10"/>
         <v>5.6611578157504416</v>
       </c>
-      <c r="N78">
-        <f t="shared" si="10"/>
+      <c r="N87">
+        <f t="shared" si="11"/>
         <v>20.380168136701592</v>
       </c>
-      <c r="O78">
-        <f t="shared" si="11"/>
+      <c r="O87">
+        <f t="shared" si="12"/>
         <v>-79.619831863298401</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A79">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A88">
         <v>3900.03</v>
       </c>
-      <c r="B79">
+      <c r="B88">
         <v>31006</v>
       </c>
-      <c r="C79">
+      <c r="C88">
         <v>50</v>
       </c>
-      <c r="D79" t="s">
-        <v>30</v>
-      </c>
-      <c r="E79" s="1">
+      <c r="D88" t="s">
+        <v>17</v>
+      </c>
+      <c r="E88" s="1">
         <v>31006</v>
       </c>
-      <c r="G79">
+      <c r="F88">
+        <f t="shared" si="17"/>
         <v>139.69999999999999</v>
       </c>
-      <c r="H79">
+      <c r="G88">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="H88">
         <v>2</v>
       </c>
-      <c r="I79">
-        <f t="shared" si="6"/>
+      <c r="I88">
+        <f t="shared" si="7"/>
         <v>0.13569999999999999</v>
       </c>
-      <c r="J79">
-        <f t="shared" si="7"/>
-        <v>1.4462706625900674E-2</v>
-      </c>
-      <c r="K79">
-        <v>1</v>
-      </c>
-      <c r="L79">
+      <c r="J88">
         <f t="shared" si="8"/>
         <v>1.4462706625900674E-2</v>
       </c>
-      <c r="M79">
+      <c r="K88">
+        <v>1</v>
+      </c>
+      <c r="L88">
         <f t="shared" si="9"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="M88">
+        <f t="shared" si="10"/>
         <v>14.462706625900674</v>
       </c>
-      <c r="N79">
-        <f t="shared" si="10"/>
+      <c r="N88">
+        <f t="shared" si="11"/>
         <v>52.065743853242424</v>
       </c>
-      <c r="O79">
-        <f t="shared" si="11"/>
+      <c r="O88">
+        <f t="shared" si="12"/>
         <v>2.0657438532424237</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A80">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A89">
         <v>3900.03</v>
       </c>
-      <c r="B80">
+      <c r="B89">
         <v>3906</v>
       </c>
-      <c r="C80">
+      <c r="C89">
         <v>50</v>
       </c>
-      <c r="D80" t="s">
-        <v>31</v>
-      </c>
-      <c r="E80" s="1">
+      <c r="D89" t="s">
+        <v>17</v>
+      </c>
+      <c r="E89" s="1">
         <v>3906</v>
       </c>
-      <c r="G80">
+      <c r="F89">
+        <f t="shared" si="17"/>
         <v>139.69999999999999</v>
       </c>
-      <c r="H80">
+      <c r="G89">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="H89">
         <v>2</v>
       </c>
-      <c r="I80">
-        <f t="shared" si="6"/>
+      <c r="I89">
+        <f t="shared" si="7"/>
         <v>0.13569999999999999</v>
       </c>
-      <c r="J80">
-        <f t="shared" si="7"/>
-        <v>1.4462706625900674E-2</v>
-      </c>
-      <c r="K80">
-        <v>1</v>
-      </c>
-      <c r="L80">
+      <c r="J89">
         <f t="shared" si="8"/>
         <v>1.4462706625900674E-2</v>
       </c>
-      <c r="M80">
+      <c r="K89">
+        <v>1</v>
+      </c>
+      <c r="L89">
         <f t="shared" si="9"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="M89">
+        <f t="shared" si="10"/>
         <v>14.462706625900674</v>
       </c>
-      <c r="N80">
-        <f t="shared" si="10"/>
+      <c r="N89">
+        <f t="shared" si="11"/>
         <v>52.065743853242424</v>
       </c>
-      <c r="O80">
-        <f t="shared" si="11"/>
+      <c r="O89">
+        <f t="shared" si="12"/>
         <v>2.0657438532424237</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A81">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A90">
         <v>19</v>
       </c>
-      <c r="B81">
+      <c r="B90">
         <v>3800.01</v>
       </c>
-      <c r="C81">
+      <c r="C90">
         <v>120</v>
       </c>
-      <c r="D81" t="s">
-        <v>32</v>
-      </c>
-      <c r="E81" s="1">
+      <c r="D90" t="s">
+        <v>18</v>
+      </c>
+      <c r="E90" s="1">
         <v>3800.01</v>
       </c>
-      <c r="G81">
+      <c r="F90">
+        <f t="shared" si="17"/>
         <v>155</v>
       </c>
-      <c r="H81">
+      <c r="G90">
+        <v>155</v>
+      </c>
+      <c r="H90">
         <v>2</v>
       </c>
-      <c r="I81">
-        <f t="shared" si="6"/>
+      <c r="I90">
+        <f t="shared" si="7"/>
         <v>0.151</v>
       </c>
-      <c r="J81">
-        <f t="shared" si="7"/>
-        <v>1.7907863523625216E-2</v>
-      </c>
-      <c r="K81">
-        <v>1</v>
-      </c>
-      <c r="L81">
+      <c r="J90">
         <f t="shared" si="8"/>
         <v>1.7907863523625216E-2</v>
       </c>
-      <c r="M81">
+      <c r="K90">
+        <v>1</v>
+      </c>
+      <c r="L90">
         <f t="shared" si="9"/>
+        <v>1.7907863523625216E-2</v>
+      </c>
+      <c r="M90">
+        <f t="shared" si="10"/>
         <v>17.907863523625217</v>
       </c>
-      <c r="N81">
-        <f t="shared" si="10"/>
+      <c r="N90">
+        <f t="shared" si="11"/>
         <v>64.468308685050772</v>
       </c>
-      <c r="O81">
-        <f t="shared" si="11"/>
+      <c r="O90">
+        <f t="shared" si="12"/>
         <v>-55.531691314949228</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A82">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A91">
         <v>3800.01</v>
       </c>
-      <c r="B82">
+      <c r="B91">
         <v>3801</v>
       </c>
-      <c r="C82">
+      <c r="C91">
         <v>90</v>
       </c>
-      <c r="D82" t="s">
-        <v>33</v>
-      </c>
-      <c r="E82" s="1">
+      <c r="D91" t="s">
+        <v>18</v>
+      </c>
+      <c r="E91" s="1">
         <v>3801</v>
       </c>
-      <c r="G82">
+      <c r="F91">
+        <f t="shared" si="17"/>
         <v>88.9</v>
       </c>
-      <c r="H82">
+      <c r="G91">
+        <v>88.9</v>
+      </c>
+      <c r="H91">
         <v>2</v>
       </c>
-      <c r="I82">
-        <f t="shared" si="6"/>
+      <c r="I91">
+        <f t="shared" si="7"/>
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="J82">
-        <f t="shared" si="7"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="K82">
-        <v>1</v>
-      </c>
-      <c r="L82">
+      <c r="J91">
         <f t="shared" si="8"/>
         <v>5.661157815750442E-3</v>
       </c>
-      <c r="M82">
+      <c r="K91">
+        <v>1</v>
+      </c>
+      <c r="L91">
         <f t="shared" si="9"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="M91">
+        <f t="shared" si="10"/>
         <v>5.6611578157504416</v>
       </c>
-      <c r="N82">
-        <f t="shared" si="10"/>
+      <c r="N91">
+        <f t="shared" si="11"/>
         <v>20.380168136701592</v>
       </c>
-      <c r="O82">
-        <f t="shared" si="11"/>
+      <c r="O91">
+        <f t="shared" si="12"/>
         <v>-69.619831863298401</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A83">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A92">
         <v>3800.01</v>
       </c>
-      <c r="B83">
+      <c r="B92">
         <v>3806</v>
       </c>
-      <c r="C83">
+      <c r="C92">
         <v>30</v>
       </c>
-      <c r="D83" t="s">
-        <v>34</v>
-      </c>
-      <c r="E83" s="1">
+      <c r="D92" t="s">
+        <v>18</v>
+      </c>
+      <c r="E92" s="1">
         <v>3806</v>
       </c>
-      <c r="G83">
+      <c r="F92">
+        <f t="shared" si="17"/>
         <v>139.69999999999999</v>
       </c>
-      <c r="H83">
+      <c r="G92">
+        <v>139.69999999999999</v>
+      </c>
+      <c r="H92">
         <v>2</v>
       </c>
-      <c r="I83">
-        <f t="shared" si="6"/>
+      <c r="I92">
+        <f t="shared" si="7"/>
         <v>0.13569999999999999</v>
       </c>
-      <c r="J83">
-        <f t="shared" si="7"/>
-        <v>1.4462706625900674E-2</v>
-      </c>
-      <c r="K83">
-        <v>1</v>
-      </c>
-      <c r="L83">
+      <c r="J92">
         <f t="shared" si="8"/>
         <v>1.4462706625900674E-2</v>
       </c>
-      <c r="M83">
+      <c r="K92">
+        <v>1</v>
+      </c>
+      <c r="L92">
         <f t="shared" si="9"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="M92">
+        <f t="shared" si="10"/>
         <v>14.462706625900674</v>
       </c>
-      <c r="N83">
-        <f t="shared" si="10"/>
+      <c r="N92">
+        <f t="shared" si="11"/>
         <v>52.065743853242424</v>
       </c>
-      <c r="O83">
-        <f t="shared" si="11"/>
+      <c r="O92">
+        <f t="shared" si="12"/>
         <v>22.065743853242424</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A84">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A93">
         <v>20</v>
       </c>
-      <c r="B84">
+      <c r="B93">
         <v>4200.01</v>
       </c>
-      <c r="C84">
+      <c r="C93">
         <v>20</v>
       </c>
-      <c r="D84" t="s">
-        <v>35</v>
-      </c>
-      <c r="E84" s="1">
+      <c r="D93" t="s">
+        <v>19</v>
+      </c>
+      <c r="E93" s="1">
         <v>4200.01</v>
       </c>
-      <c r="F84">
+      <c r="F93">
         <v>100</v>
       </c>
-      <c r="G84">
+      <c r="G93">
         <v>114</v>
       </c>
-      <c r="H84">
+      <c r="H93">
         <v>4.5</v>
       </c>
-      <c r="I84">
-        <f t="shared" si="6"/>
+      <c r="I93">
+        <f t="shared" si="7"/>
         <v>0.105</v>
       </c>
-      <c r="J84">
-        <f t="shared" si="7"/>
-        <v>8.6590147514568668E-3</v>
-      </c>
-      <c r="K84">
-        <v>1</v>
-      </c>
-      <c r="L84">
+      <c r="J93">
         <f t="shared" si="8"/>
         <v>8.6590147514568668E-3</v>
       </c>
-      <c r="M84">
+      <c r="K93">
+        <v>1</v>
+      </c>
+      <c r="L93">
         <f t="shared" si="9"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="M93">
+        <f t="shared" si="10"/>
         <v>8.6590147514568674</v>
       </c>
-      <c r="N84">
-        <f t="shared" si="10"/>
+      <c r="N93">
+        <f t="shared" si="11"/>
         <v>31.17245310524472</v>
       </c>
-      <c r="O84">
-        <f t="shared" si="11"/>
+      <c r="O93">
+        <f t="shared" si="12"/>
         <v>11.17245310524472</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A85">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A94">
         <v>4200.01</v>
       </c>
-      <c r="B85">
+      <c r="B94">
         <v>4202</v>
       </c>
-      <c r="C85">
+      <c r="C94">
         <v>10</v>
       </c>
-      <c r="D85" t="s">
-        <v>35</v>
-      </c>
-      <c r="E85" s="1">
+      <c r="D94" t="s">
+        <v>19</v>
+      </c>
+      <c r="E94" s="1">
         <v>4202</v>
       </c>
-      <c r="F85">
+      <c r="F94">
         <v>65</v>
       </c>
-      <c r="G85">
+      <c r="G94">
         <v>76.099999999999994</v>
       </c>
-      <c r="H85">
+      <c r="H94">
         <v>3.6</v>
       </c>
-      <c r="I85">
-        <f t="shared" si="6"/>
+      <c r="I94">
+        <f t="shared" si="7"/>
         <v>6.8899999999999989E-2</v>
       </c>
-      <c r="J85">
-        <f t="shared" si="7"/>
-        <v>3.728450015261999E-3</v>
-      </c>
-      <c r="K85">
-        <v>1</v>
-      </c>
-      <c r="L85">
+      <c r="J94">
         <f t="shared" si="8"/>
         <v>3.728450015261999E-3</v>
       </c>
-      <c r="M85">
+      <c r="K94">
+        <v>1</v>
+      </c>
+      <c r="L94">
         <f t="shared" si="9"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M94">
+        <f t="shared" si="10"/>
         <v>3.7284500152619988</v>
       </c>
-      <c r="N85">
-        <f t="shared" si="10"/>
+      <c r="N94">
+        <f t="shared" si="11"/>
         <v>13.422420054943197</v>
       </c>
-      <c r="O85">
-        <f t="shared" si="11"/>
+      <c r="O94">
+        <f t="shared" si="12"/>
         <v>3.4224200549431973</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A86">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A95">
         <v>4200.01</v>
       </c>
-      <c r="B86">
+      <c r="B95">
         <v>4201</v>
       </c>
-      <c r="C86">
+      <c r="C95">
         <v>10</v>
       </c>
-      <c r="D86" t="s">
-        <v>35</v>
-      </c>
-      <c r="E86" s="1">
+      <c r="D95" t="s">
+        <v>19</v>
+      </c>
+      <c r="E95" s="1">
         <v>4201</v>
       </c>
-      <c r="F86">
+      <c r="F95">
         <v>65</v>
       </c>
-      <c r="G86">
+      <c r="G95">
         <v>76.099999999999994</v>
       </c>
-      <c r="H86">
+      <c r="H95">
         <v>3.6</v>
       </c>
-      <c r="I86">
-        <f t="shared" si="6"/>
+      <c r="I95">
+        <f t="shared" si="7"/>
         <v>6.8899999999999989E-2</v>
       </c>
-      <c r="J86">
-        <f t="shared" si="7"/>
-        <v>3.728450015261999E-3</v>
-      </c>
-      <c r="K86">
-        <v>1</v>
-      </c>
-      <c r="L86">
+      <c r="J95">
         <f t="shared" si="8"/>
         <v>3.728450015261999E-3</v>
       </c>
-      <c r="M86">
+      <c r="K95">
+        <v>1</v>
+      </c>
+      <c r="L95">
         <f t="shared" si="9"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M95">
+        <f t="shared" si="10"/>
         <v>3.7284500152619988</v>
       </c>
-      <c r="N86">
-        <f t="shared" si="10"/>
+      <c r="N95">
+        <f t="shared" si="11"/>
         <v>13.422420054943197</v>
       </c>
-      <c r="O86">
-        <f t="shared" si="11"/>
+      <c r="O95">
+        <f t="shared" si="12"/>
         <v>3.4224200549431973</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A87">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A96">
         <v>21</v>
       </c>
-      <c r="B87">
+      <c r="B96">
         <v>4300.01</v>
       </c>
-      <c r="C87">
+      <c r="C96">
         <v>10</v>
       </c>
-      <c r="D87" t="s">
-        <v>35</v>
-      </c>
-      <c r="E87" s="1">
+      <c r="D96" t="s">
+        <v>19</v>
+      </c>
+      <c r="E96" s="1">
         <v>4300.01</v>
       </c>
-      <c r="F87">
+      <c r="F96">
         <v>65</v>
       </c>
-      <c r="G87">
+      <c r="G96">
         <v>76.099999999999994</v>
       </c>
-      <c r="H87">
+      <c r="H96">
         <v>3.6</v>
       </c>
-      <c r="I87">
-        <f t="shared" si="6"/>
+      <c r="I96">
+        <f t="shared" si="7"/>
         <v>6.8899999999999989E-2</v>
       </c>
-      <c r="J87">
-        <f t="shared" si="7"/>
-        <v>3.728450015261999E-3</v>
-      </c>
-      <c r="K87">
-        <v>1</v>
-      </c>
-      <c r="L87">
+      <c r="J96">
         <f t="shared" si="8"/>
         <v>3.728450015261999E-3</v>
       </c>
-      <c r="M87">
+      <c r="K96">
+        <v>1</v>
+      </c>
+      <c r="L96">
         <f t="shared" si="9"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="M96">
+        <f t="shared" si="10"/>
         <v>3.7284500152619988</v>
       </c>
-      <c r="N87">
-        <f t="shared" si="10"/>
+      <c r="N96">
+        <f t="shared" si="11"/>
         <v>13.422420054943197</v>
       </c>
-      <c r="O87">
-        <f t="shared" si="11"/>
+      <c r="O96">
+        <f t="shared" si="12"/>
         <v>3.4224200549431973</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A88">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A97">
         <v>4300.01</v>
       </c>
-      <c r="B88">
+      <c r="B97">
         <v>4303</v>
       </c>
-      <c r="C88">
+      <c r="C97">
         <v>5</v>
       </c>
-      <c r="D88" t="s">
-        <v>35</v>
-      </c>
-      <c r="E88" s="1">
+      <c r="D97" t="s">
+        <v>19</v>
+      </c>
+      <c r="E97" s="1">
         <v>4303</v>
       </c>
-      <c r="F88">
+      <c r="F97">
         <v>50</v>
       </c>
-      <c r="G88">
+      <c r="G97">
         <v>60.3</v>
       </c>
-      <c r="H88">
+      <c r="H97">
         <v>3.6</v>
       </c>
-      <c r="I88">
-        <f t="shared" si="6"/>
+      <c r="I97">
+        <f t="shared" si="7"/>
         <v>5.3099999999999994E-2</v>
       </c>
-      <c r="J88">
-        <f t="shared" si="7"/>
-        <v>2.2145165154970788E-3</v>
-      </c>
-      <c r="K88">
-        <v>1</v>
-      </c>
-      <c r="L88">
+      <c r="J97">
         <f t="shared" si="8"/>
         <v>2.2145165154970788E-3</v>
       </c>
-      <c r="M88">
+      <c r="K97">
+        <v>1</v>
+      </c>
+      <c r="L97">
         <f t="shared" si="9"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M97">
+        <f t="shared" si="10"/>
         <v>2.214516515497079</v>
       </c>
-      <c r="N88">
-        <f t="shared" si="10"/>
+      <c r="N97">
+        <f t="shared" si="11"/>
         <v>7.9722594557894837</v>
       </c>
-      <c r="O88">
-        <f t="shared" si="11"/>
+      <c r="O97">
+        <f t="shared" si="12"/>
         <v>2.9722594557894837</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A89">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A98">
         <v>4300.01</v>
       </c>
-      <c r="B89">
+      <c r="B98">
         <v>4304</v>
       </c>
-      <c r="C89">
+      <c r="C98">
         <v>5</v>
       </c>
-      <c r="D89" t="s">
-        <v>35</v>
-      </c>
-      <c r="E89" s="1">
+      <c r="D98" t="s">
+        <v>19</v>
+      </c>
+      <c r="E98" s="1">
         <v>4304</v>
       </c>
-      <c r="F89">
+      <c r="F98">
         <v>50</v>
       </c>
-      <c r="G89">
+      <c r="G98">
         <v>60.3</v>
       </c>
-      <c r="H89">
+      <c r="H98">
         <v>3.6</v>
       </c>
-      <c r="I89">
-        <f t="shared" si="6"/>
+      <c r="I98">
+        <f t="shared" si="7"/>
         <v>5.3099999999999994E-2</v>
       </c>
-      <c r="J89">
-        <f t="shared" si="7"/>
-        <v>2.2145165154970788E-3</v>
-      </c>
-      <c r="K89">
-        <v>1</v>
-      </c>
-      <c r="L89">
+      <c r="J98">
         <f t="shared" si="8"/>
         <v>2.2145165154970788E-3</v>
       </c>
-      <c r="M89">
+      <c r="K98">
+        <v>1</v>
+      </c>
+      <c r="L98">
         <f t="shared" si="9"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="M98">
+        <f t="shared" si="10"/>
         <v>2.214516515497079</v>
       </c>
-      <c r="N89">
-        <f t="shared" si="10"/>
+      <c r="N98">
+        <f t="shared" si="11"/>
         <v>7.9722594557894837</v>
       </c>
-      <c r="O89">
-        <f t="shared" si="11"/>
+      <c r="O98">
+        <f t="shared" si="12"/>
         <v>2.9722594557894837</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>